<commit_message>
criado o check list do profile
</commit_message>
<xml_diff>
--- a/doc/profiles_list.xlsx
+++ b/doc/profiles_list.xlsx
@@ -28,25 +28,25 @@
     <t xml:space="preserve">TELEGRAM_ALLOWED_USERS</t>
   </si>
   <si>
-    <t xml:space="preserve">Bot name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descrição (opcional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Username</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Profile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Token</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TELEGRAM_HOME_CHANNEL_NAME </t>
-  </si>
-  <si>
-    <t xml:space="preserve">NAME</t>
+    <t xml:space="preserve">BOT_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USERNAME_BOT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROFILE_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOT_TOKEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome do bot no Chat </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome do bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome do profile no Hermes</t>
   </si>
   <si>
     <t xml:space="preserve">TELEGRAM_BOT_TOKEN</t>
@@ -91,9 +91,10 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="10"/>
+      <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -157,7 +158,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -352,14 +353,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.69"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -384,23 +384,21 @@
       <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="2" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="D5" s="4" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>